<commit_message>
Engine: math.fsum for all float sums so results are bit-identical across Python versions
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018QDEZA5PJVsN59HaHx5Eer
</commit_message>
<xml_diff>
--- a/results/alternatives/P1_earth_only_BASE/results.xlsx
+++ b/results/alternatives/P1_earth_only_BASE/results.xlsx
@@ -1423,19 +1423,19 @@
         <v>80</v>
       </c>
       <c r="F2" t="n">
-        <v>99.99999999999999</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
         <v>80</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>1.4210854715202e-14</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -1456,7 +1456,7 @@
         <v>4.944420000000001</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.045</v>
+        <v>0.04500000000000001</v>
       </c>
       <c r="R2" t="n">
         <v>12.32876712328767</v>
@@ -1479,7 +1479,7 @@
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>7.105427357601002e-15</v>
+        <v>-3.552713678800501e-14</v>
       </c>
     </row>
     <row r="3">
@@ -1533,7 +1533,7 @@
         <v>153.0518</v>
       </c>
       <c r="P3" t="n">
-        <v>6.887331000000001</v>
+        <v>6.887331</v>
       </c>
       <c r="Q3" t="n">
         <v>0.04500000000000001</v>
@@ -1613,7 +1613,7 @@
         <v>206.6988</v>
       </c>
       <c r="P4" t="n">
-        <v>9.301446</v>
+        <v>9.301446000000002</v>
       </c>
       <c r="Q4" t="n">
         <v>0.04500000000000001</v>
@@ -1625,7 +1625,7 @@
         <v>1</v>
       </c>
       <c r="T4" t="n">
-        <v>27.12358500000006</v>
+        <v>27.12358500000005</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>-7.105427357601002e-15</v>
+        <v>4.973799150320701e-14</v>
       </c>
     </row>
     <row r="5">
@@ -1719,7 +1719,7 @@
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>-4.263256414560601e-14</v>
+        <v>4.263256414560601e-14</v>
       </c>
     </row>
     <row r="6">
@@ -1785,7 +1785,7 @@
         <v>1</v>
       </c>
       <c r="T6" t="n">
-        <v>22.70240149999999</v>
+        <v>22.7024015</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -1826,7 +1826,7 @@
         <v>292.4524015</v>
       </c>
       <c r="G7" t="n">
-        <v>250.0000000000001</v>
+        <v>250</v>
       </c>
       <c r="H7" t="n">
         <v>0.7498779525641024</v>
@@ -8184,10 +8184,10 @@
         <v>16.6988</v>
       </c>
       <c r="M14" t="n">
-        <v>16.69879999999999</v>
+        <v>16.6988</v>
       </c>
       <c r="N14" t="n">
-        <v>16.69879999999999</v>
+        <v>16.6988</v>
       </c>
       <c r="O14" t="n">
         <v>1</v>
@@ -8559,10 +8559,10 @@
         <v>80.8169</v>
       </c>
       <c r="M19" t="n">
-        <v>80.81689999999999</v>
+        <v>80.8169</v>
       </c>
       <c r="N19" t="n">
-        <v>80.81689999999999</v>
+        <v>80.8169</v>
       </c>
       <c r="O19" t="n">
         <v>1</v>
@@ -10407,7 +10407,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>0.97</v>
@@ -20317,7 +20317,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>950.0000000000001</v>
+        <v>950</v>
       </c>
     </row>
     <row r="8">
@@ -20337,7 +20337,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>97.54759850000006</v>
+        <v>97.54759850000005</v>
       </c>
     </row>
     <row r="9">

</xml_diff>